<commit_message>
Alternate link added for ESP-PSRAM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark-BOM-v2.0 Boards.xlsx
+++ b/Deliverables/BOM/eSpark-BOM-v2.0 Boards.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Melih-SoundSensor\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\Melih-SoundSensor\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E4CAA0-8330-4AE9-90D8-95D5EB6C7219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6780" yWindow="3075" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-6780" yWindow="3075" windowWidth="11790" windowHeight="15360"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="301">
   <si>
     <t>S. No.</t>
   </si>
@@ -936,12 +935,15 @@
   </si>
   <si>
     <t>Total with Shipping Single Board</t>
+  </si>
+  <si>
+    <t>Alternate Supplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
@@ -1690,7 +1692,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="274">
+  <cellXfs count="275">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2497,6 +2499,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2774,7 +2779,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:W68"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -5562,8 +5567,8 @@
         <v>30</v>
       </c>
       <c r="U41" s="165"/>
-      <c r="V41" s="148" t="s">
-        <v>291</v>
+      <c r="V41" s="274" t="s">
+        <v>300</v>
       </c>
       <c r="W41" s="149"/>
     </row>
@@ -6543,52 +6548,53 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="P3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="P4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="P5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="P6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="P8" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="P9" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="P10" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="P11" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="P25" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="P26" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="P27" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="P29" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="P33" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="P35" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="P42" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="P43" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="P45" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="P24" r:id="rId18" display="Aliexpress" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="P44" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="P7" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="P12" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="P13" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="P18" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="P20" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="P28" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="P31" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="P38" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="P39" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="P14" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="P15" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="P32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="P50" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="P49" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="P16" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="P17" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="P30" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="P46" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="P41" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="P47" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="P19" r:id="rId40" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="P40" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="P23" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="P22" r:id="rId43" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="P3" r:id="rId1"/>
+    <hyperlink ref="P4" r:id="rId2"/>
+    <hyperlink ref="P5" r:id="rId3"/>
+    <hyperlink ref="P6" r:id="rId4"/>
+    <hyperlink ref="P8" r:id="rId5"/>
+    <hyperlink ref="P9" r:id="rId6"/>
+    <hyperlink ref="P10" r:id="rId7"/>
+    <hyperlink ref="P11" r:id="rId8"/>
+    <hyperlink ref="P25" r:id="rId9"/>
+    <hyperlink ref="P26" r:id="rId10"/>
+    <hyperlink ref="P27" r:id="rId11"/>
+    <hyperlink ref="P29" r:id="rId12"/>
+    <hyperlink ref="P33" r:id="rId13"/>
+    <hyperlink ref="P35" r:id="rId14"/>
+    <hyperlink ref="P42" r:id="rId15"/>
+    <hyperlink ref="P43" r:id="rId16"/>
+    <hyperlink ref="P45" r:id="rId17"/>
+    <hyperlink ref="P24" r:id="rId18" display="Aliexpress"/>
+    <hyperlink ref="P44" r:id="rId19"/>
+    <hyperlink ref="P7" r:id="rId20"/>
+    <hyperlink ref="P12" r:id="rId21"/>
+    <hyperlink ref="P13" r:id="rId22"/>
+    <hyperlink ref="P18" r:id="rId23"/>
+    <hyperlink ref="P20" r:id="rId24"/>
+    <hyperlink ref="P28" r:id="rId25"/>
+    <hyperlink ref="P31" r:id="rId26"/>
+    <hyperlink ref="P38" r:id="rId27"/>
+    <hyperlink ref="P39" r:id="rId28"/>
+    <hyperlink ref="P14" r:id="rId29"/>
+    <hyperlink ref="P15" r:id="rId30"/>
+    <hyperlink ref="P32" r:id="rId31"/>
+    <hyperlink ref="P50" r:id="rId32"/>
+    <hyperlink ref="P49" r:id="rId33"/>
+    <hyperlink ref="P16" r:id="rId34"/>
+    <hyperlink ref="P17" r:id="rId35"/>
+    <hyperlink ref="P30" r:id="rId36"/>
+    <hyperlink ref="P46" r:id="rId37"/>
+    <hyperlink ref="P41" r:id="rId38"/>
+    <hyperlink ref="P47" r:id="rId39"/>
+    <hyperlink ref="P19" r:id="rId40"/>
+    <hyperlink ref="P40" r:id="rId41"/>
+    <hyperlink ref="P23" r:id="rId42"/>
+    <hyperlink ref="P22" r:id="rId43"/>
+    <hyperlink ref="V41" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId44"/>
+  <pageSetup orientation="portrait" r:id="rId45"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>

</xml_diff>